<commit_message>
Actualización de documentos + Informe oficial del proyecto - Jaime Vergara
</commit_message>
<xml_diff>
--- a/documentos/Historias_Usuario_Martech.xls.xlsx
+++ b/documentos/Historias_Usuario_Martech.xls.xlsx
@@ -17,19 +17,19 @@
     <t>Historias de usuario y criterios de aceptación: Instructivo</t>
   </si>
   <si>
+    <t>Elaborado por: www.pmoinformatica.com</t>
+  </si>
+  <si>
+    <t>Columna</t>
+  </si>
+  <si>
+    <t>Instrucciones</t>
+  </si>
+  <si>
+    <t>Identificador (ID) de la historia</t>
+  </si>
+  <si>
     <t>Desarrollo ágil: Historias de usuario y criterios de aceptación</t>
-  </si>
-  <si>
-    <t>Elaborado por: www.pmoinformatica.com</t>
-  </si>
-  <si>
-    <t>Columna</t>
-  </si>
-  <si>
-    <t>Instrucciones</t>
-  </si>
-  <si>
-    <t>Identificador (ID) de la historia</t>
   </si>
   <si>
     <t>Código que identifica unívocamente a la historia en el Proyecto que se esté desarrollando. El formato debe ser elegido por el equipo.</t>
@@ -60,42 +60,42 @@
     <t>Lo que el rol necesita lograr al ejecutar la acción. Este es el resultado de ejecutar la acción desde el punto de vista del rol. Este punto puede ser opcional, pues la historia puede documentarse sólo con la definición del rol y la acción (sin definir la consecuencia).</t>
   </si>
   <si>
+    <t>Número (#) de Escenario</t>
+  </si>
+  <si>
+    <t>Número (ejemplo 1, 2, 3 ó 4), que identifica al escenario asociado a la historia.</t>
+  </si>
+  <si>
+    <t>Criterio de Aceptación (Título)</t>
+  </si>
+  <si>
+    <t>Describe el contexto del escenario que define un comportamiento. Por ejemplo, si se toma el ejemplo de búsquedas de productos por categoría, un posible ejemplo pudiera ser: Categoría sin productos asociados.</t>
+  </si>
+  <si>
+    <t>Contexto</t>
+  </si>
+  <si>
+    <t>Proporciona mayor descripción sobre las condiciones que desencadenan el escenario.</t>
+  </si>
+  <si>
+    <t>Evento</t>
+  </si>
+  <si>
+    <t>Representa la acción que el usuario ejecuta, en el contexto definido para el escenario.</t>
+  </si>
+  <si>
+    <t>Resultado / Comportamiento esperado</t>
+  </si>
+  <si>
+    <t>Dado el contexto y la acción ejecutada por el usuario, la consecuencia es el comportamiento del sistema en esa situación.</t>
+  </si>
+  <si>
     <t>Enunciado de la Historia</t>
   </si>
   <si>
-    <t>Número (#) de Escenario</t>
-  </si>
-  <si>
-    <t>Número (ejemplo 1, 2, 3 ó 4), que identifica al escenario asociado a la historia.</t>
-  </si>
-  <si>
-    <t>Criterio de Aceptación (Título)</t>
-  </si>
-  <si>
-    <t>Describe el contexto del escenario que define un comportamiento. Por ejemplo, si se toma el ejemplo de búsquedas de productos por categoría, un posible ejemplo pudiera ser: Categoría sin productos asociados.</t>
-  </si>
-  <si>
-    <t>Contexto</t>
-  </si>
-  <si>
-    <t>Proporciona mayor descripción sobre las condiciones que desencadenan el escenario.</t>
-  </si>
-  <si>
     <t>Criterios de Aceptación</t>
   </si>
   <si>
-    <t>Evento</t>
-  </si>
-  <si>
-    <t>Representa la acción que el usuario ejecuta, en el contexto definido para el escenario.</t>
-  </si>
-  <si>
-    <t>Resultado / Comportamiento esperado</t>
-  </si>
-  <si>
-    <t>Dado el contexto y la acción ejecutada por el usuario, la consecuencia es el comportamiento del sistema en esa situación.</t>
-  </si>
-  <si>
     <t>Identificador (ID) de la Historia</t>
   </si>
   <si>
@@ -918,7 +918,7 @@
     <t>Necesito Consultar los resultados de los trabajos llevados a cabo por las diferentes herramientas de automatización que se usen a lo largo del tratamiento de los datos además de los propios datos después de cada una de sus transformaciones.</t>
   </si>
   <si>
-    <t>Para realizar un seguimiento de desempeño y verificación de los cambios aplicados a os propios datos.</t>
+    <t>Para realizar un seguimiento de desempeño y verificación de los cambios aplicados a los propios datos.</t>
   </si>
   <si>
     <t>Consulta de trazabilidad de ejecución</t>
@@ -1284,12 +1284,6 @@
     </font>
     <font>
       <b/>
-      <sz val="28.0"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
       <sz val="16.0"/>
       <color rgb="FF1F497D"/>
       <name val="Calibri"/>
@@ -1297,6 +1291,12 @@
     <font>
       <sz val="11.0"/>
       <color theme="0"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="28.0"/>
+      <color theme="1"/>
       <name val="Calibri"/>
     </font>
     <font/>
@@ -1456,22 +1456,22 @@
     <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="2" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="2" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="2" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
+    <xf borderId="1" fillId="2" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
     <xf borderId="3" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="3" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="3" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="4" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="6" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
@@ -1482,7 +1482,7 @@
     <xf borderId="2" fillId="3" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="2" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="2" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="8" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
@@ -1761,8 +1761,8 @@
   <sheetData>
     <row r="1" ht="36.0" customHeight="1">
       <c r="A1" s="1"/>
-      <c r="B1" s="3" t="s">
-        <v>1</v>
+      <c r="B1" s="6" t="s">
+        <v>5</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -1793,7 +1793,7 @@
     </row>
     <row r="2" ht="21.0" customHeight="1">
       <c r="A2" s="1"/>
-      <c r="B2" s="4"/>
+      <c r="B2" s="3"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -1857,13 +1857,13 @@
       <c r="C4" s="8"/>
       <c r="D4" s="8"/>
       <c r="E4" s="9" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="F4" s="10"/>
       <c r="G4" s="10"/>
       <c r="H4" s="11"/>
       <c r="I4" s="9" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="J4" s="10"/>
       <c r="K4" s="10"/>
@@ -1906,19 +1906,19 @@
         <v>11</v>
       </c>
       <c r="H5" s="13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I5" s="13" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J5" s="13" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="K5" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="L5" s="13" t="s">
         <v>21</v>
-      </c>
-      <c r="L5" s="13" t="s">
-        <v>23</v>
       </c>
       <c r="M5" s="15"/>
       <c r="N5" s="1"/>
@@ -10448,8 +10448,8 @@
     </row>
     <row r="2" ht="21.0" customHeight="1">
       <c r="A2" s="1"/>
-      <c r="B2" s="4" t="s">
-        <v>2</v>
+      <c r="B2" s="3" t="s">
+        <v>1</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -10506,11 +10506,11 @@
     </row>
     <row r="4">
       <c r="A4" s="1"/>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>3</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>4</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
@@ -10538,10 +10538,10 @@
     </row>
     <row r="5" ht="30.0" customHeight="1">
       <c r="A5" s="1"/>
-      <c r="B5" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5" s="6" t="s">
+      <c r="B5" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>6</v>
       </c>
       <c r="D5" s="1"/>
@@ -10570,10 +10570,10 @@
     </row>
     <row r="6" ht="135.0" customHeight="1">
       <c r="A6" s="1"/>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="5" t="s">
         <v>8</v>
       </c>
       <c r="D6" s="1"/>
@@ -10602,10 +10602,10 @@
     </row>
     <row r="7" ht="105.0" customHeight="1">
       <c r="A7" s="1"/>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="5" t="s">
         <v>10</v>
       </c>
       <c r="D7" s="1"/>
@@ -10634,10 +10634,10 @@
     </row>
     <row r="8" ht="45.0" customHeight="1">
       <c r="A8" s="1"/>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="5" t="s">
         <v>12</v>
       </c>
       <c r="D8" s="1"/>
@@ -10666,11 +10666,11 @@
     </row>
     <row r="9">
       <c r="A9" s="1"/>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" s="5" t="s">
         <v>14</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>15</v>
       </c>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
@@ -10698,11 +10698,11 @@
     </row>
     <row r="10" ht="45.0" customHeight="1">
       <c r="A10" s="1"/>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" s="5" t="s">
         <v>16</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>17</v>
       </c>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
@@ -10730,11 +10730,11 @@
     </row>
     <row r="11">
       <c r="A11" s="1"/>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>18</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>19</v>
       </c>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
@@ -10762,11 +10762,11 @@
     </row>
     <row r="12">
       <c r="A12" s="1"/>
-      <c r="B12" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>22</v>
+      <c r="B12" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>20</v>
       </c>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
@@ -10794,11 +10794,11 @@
     </row>
     <row r="13" ht="30.0" customHeight="1">
       <c r="A13" s="1"/>
-      <c r="B13" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>24</v>
+      <c r="B13" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>22</v>
       </c>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>

</xml_diff>